<commit_message>
Fix: course detail redirecting to login for non-enrolled users
Backend: Return empty assignments list instead of 401 for non-enrolled
users viewing a course. Students should see course details freely —
assignments are just hidden until they enroll.

Frontend: Don't redirect to /login on 401 if user has a valid token.
Only redirect when there's no token at all (actual auth failure).
This prevents permission-based 401s (enrollment checks) from
clearing the session.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Credentials/Creds.xlsx
+++ b/Credentials/Creds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Websites\Spire-Compet\Credentials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC6543B2-4346-48F0-BEA5-745A0C276C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFDDF5C0-CD20-4D32-BB9C-7AC6D5B81935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{A422E0BC-9C97-42B6-915E-A1F21E23A392}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>User</t>
   </si>
@@ -61,6 +61,18 @@
   </si>
   <si>
     <t>admin1@test.com</t>
+  </si>
+  <si>
+    <t>Roll no</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S.no </t>
+  </si>
+  <si>
+    <t>Simple</t>
+  </si>
+  <si>
+    <t>Complex</t>
   </si>
 </sst>
 </file>
@@ -428,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB622FEB-5749-4E3B-BE0C-45AC91C9E10B}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.77734375" bestFit="1" customWidth="1"/>
@@ -436,7 +448,7 @@
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -446,8 +458,20 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+      <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -457,8 +481,20 @@
       <c r="C2" s="2">
         <v>12345678</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E2">
+        <v>54</v>
+      </c>
+      <c r="F2">
+        <v>501</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -468,8 +504,20 @@
       <c r="C3">
         <v>12345678</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+      <c r="E3">
+        <v>55</v>
+      </c>
+      <c r="F3">
+        <v>502</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -478,6 +526,148 @@
       </c>
       <c r="C4" s="2">
         <v>12345678</v>
+      </c>
+      <c r="E4">
+        <v>56</v>
+      </c>
+      <c r="F4">
+        <v>503</v>
+      </c>
+      <c r="G4">
+        <v>5</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E5">
+        <v>57</v>
+      </c>
+      <c r="F5">
+        <v>504</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E6">
+        <v>58</v>
+      </c>
+      <c r="F6">
+        <v>505</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E7">
+        <v>59</v>
+      </c>
+      <c r="F7">
+        <v>506</v>
+      </c>
+      <c r="G7">
+        <v>3</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E8">
+        <v>60</v>
+      </c>
+      <c r="F8">
+        <v>507</v>
+      </c>
+      <c r="G8">
+        <v>4</v>
+      </c>
+      <c r="H8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E9">
+        <v>61</v>
+      </c>
+      <c r="F9">
+        <v>508</v>
+      </c>
+      <c r="G9">
+        <v>5</v>
+      </c>
+      <c r="H9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E10">
+        <v>62</v>
+      </c>
+      <c r="F10">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E11">
+        <v>63</v>
+      </c>
+      <c r="F11">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E12">
+        <v>64</v>
+      </c>
+      <c r="F12">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E13">
+        <v>65</v>
+      </c>
+      <c r="F13">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E14">
+        <v>66</v>
+      </c>
+      <c r="F14">
+        <v>513</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E15">
+        <v>67</v>
+      </c>
+      <c r="F15">
+        <v>514</v>
+      </c>
+      <c r="G15">
+        <v>4</v>
+      </c>
+      <c r="H15">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update color palette to match provided 4-stripe palette
Palette (top to bottom):
1. #F0EDE8 — cream/off-white (background)
2. #95C8CB — light teal/aqua (accent)
3. #5FA3A3 — medium teal (primary-light, hover states)
4. #0E6B6B — deep teal (primary, buttons, headings)

Updated: tailwind.config.ts, globals.css, layout.tsx, and all 17+
component files with hardcoded hex values.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Credentials/Creds.xlsx
+++ b/Credentials/Creds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Websites\Spire-Compet\Credentials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFDDF5C0-CD20-4D32-BB9C-7AC6D5B81935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B02D4D65-7091-4FDC-8465-8411C00C269A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{A422E0BC-9C97-42B6-915E-A1F21E23A392}"/>
   </bookViews>
@@ -666,9 +666,6 @@
       <c r="G15">
         <v>4</v>
       </c>
-      <c r="H15">
-        <v>6</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>